<commit_message>
changed to vertical connectors
</commit_message>
<xml_diff>
--- a/hardware/Scrutineering/BOM/Scrutineering.xlsx
+++ b/hardware/Scrutineering/BOM/Scrutineering.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\phoen\LHR\PS-VoltTemp\hardware\Scrutineering\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{231F4224-F0DA-4BEB-A467-4C0461C5263A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BA7F0E6-BFD0-4021-8F4C-E4F17FD36FD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{62597573-C5BD-43BE-8C8F-E66FE9158839}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="12980" windowHeight="16090" xr2:uid="{62597573-C5BD-43BE-8C8F-E66FE9158839}"/>
   </bookViews>
   <sheets>
     <sheet name="Scrutineering" sheetId="1" r:id="rId1"/>
@@ -49,15 +49,9 @@
     <t>Conn_01x03</t>
   </si>
   <si>
-    <t>VoltTemp:1053131103</t>
-  </si>
-  <si>
     <t>Conn_01x02</t>
   </si>
   <si>
-    <t>UTSVT_Connectors:105313-2102</t>
-  </si>
-  <si>
     <t>SW1,SW2,SW3,SW4</t>
   </si>
   <si>
@@ -79,13 +73,19 @@
     <t>Conn_02x04</t>
   </si>
   <si>
-    <t>Scrutineering:nanofit_02x04</t>
-  </si>
-  <si>
     <t>J3,J4</t>
   </si>
   <si>
     <t>J11,J11</t>
+  </si>
+  <si>
+    <t>UTSVT_Connectors:Molex_Nano-Fit_105309-xx02_1x02_P2.50mm_Vertical</t>
+  </si>
+  <si>
+    <t>Scrutineering:CONN_SD-105309-100_03_MOL</t>
+  </si>
+  <si>
+    <t>Scrutineering:CONN_SD-105310-100_08_MOL</t>
   </si>
 </sst>
 </file>
@@ -947,14 +947,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D2198AA-7B82-40BD-A07B-38ACB80A30FD}">
   <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.140625" customWidth="1"/>
-    <col min="2" max="2" width="13.85546875" customWidth="1"/>
-    <col min="3" max="4" width="12.140625" customWidth="1"/>
+    <col min="1" max="1" width="17.1796875" customWidth="1"/>
+    <col min="2" max="2" width="13.81640625" customWidth="1"/>
+    <col min="3" max="4" width="12.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -971,7 +971,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -979,7 +979,7 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D2" t="s">
         <v>7</v>
@@ -988,69 +988,69 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C3">
-        <v>1053132102</v>
+        <v>1053091202</v>
       </c>
       <c r="D3" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="E3">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B4" t="s">
         <v>8</v>
       </c>
       <c r="C4">
-        <v>1053131103</v>
+        <v>1053091103</v>
       </c>
       <c r="D4" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="E4">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C5">
-        <v>1053141108</v>
+        <v>1053101308</v>
       </c>
       <c r="D5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E5">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" t="s">
         <v>12</v>
-      </c>
-      <c r="B6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" t="s">
-        <v>15</v>
-      </c>
-      <c r="D6" t="s">
-        <v>14</v>
       </c>
       <c r="E6">
         <v>4</v>

</xml_diff>